<commit_message>
feat: implement analysis scripts and export pipelines for exsudat, lokalisation, and infection model performance comparison.
</commit_message>
<xml_diff>
--- a/exports/Wundtyp_Vergleich_Experten_KI.xlsx
+++ b/exports/Wundtyp_Vergleich_Experten_KI.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +41,12 @@
       <name val="Calibri"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="007F7F7F"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -125,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -151,13 +157,16 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1943,7 +1952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M65"/>
+  <dimension ref="A1:M66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -2280,9 +2289,9 @@
           <t>Postoperative Wunde / Dehiszenz</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>Prompt-Beispiel (Nicht bewertet)</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr">
@@ -2292,7 +2301,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>0/2 Uneinig</t>
+          <t>0/3 Uneinig</t>
         </is>
       </c>
     </row>
@@ -2570,22 +2579,22 @@
           <t>wunde_09</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Nekrose</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -2637,22 +2646,22 @@
           <t>wunde_10</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Dekubitus</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Dekubitus</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Dekubitus</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Dekubitus</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -2704,22 +2713,22 @@
           <t>wunde_11</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Dekubitus</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Dekubitus</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Dekubitus</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Dekubitus</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -2771,22 +2780,22 @@
           <t>wunde_12</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>Dekubitus</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Dekubitus</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -2838,22 +2847,22 @@
           <t>wunde_13</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>Dekubitus</t>
-        </is>
-      </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Dekubitus</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -2972,22 +2981,22 @@
           <t>wunde_15</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Nekrose</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -3039,22 +3048,22 @@
           <t>wunde_16</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -3173,22 +3182,22 @@
           <t>wunde_18</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -3198,9 +3207,9 @@
           <t>Traumatische Wunde</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Prompt-Beispiel (Nicht bewertet)</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -3210,7 +3219,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>0/2 Uneinig</t>
+          <t>0/3 Uneinig</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
@@ -3218,9 +3227,9 @@
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="K19" s="9" t="inlineStr">
+        <is>
+          <t>Prompt-Beispiel (Nicht bewertet)</t>
         </is>
       </c>
       <c r="L19" s="5" t="inlineStr">
@@ -3230,7 +3239,7 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>2/2 Einig</t>
+          <t>2/3 Einig</t>
         </is>
       </c>
     </row>
@@ -3240,22 +3249,22 @@
           <t>wunde_19</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>rechter Fuß lateral/ malleolär</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -3575,22 +3584,22 @@
           <t>wunde_24</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -3843,22 +3852,22 @@
           <t>wunde_28</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>Dekubitus</t>
-        </is>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>Dekubitus</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Dekubitus</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>Dekubitus</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -3868,9 +3877,9 @@
           <t>Dekubitus</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>Prompt-Beispiel (Nicht bewertet)</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -3880,7 +3889,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>2/2 Einig</t>
+          <t>2/3 Einig</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
@@ -4044,22 +4053,22 @@
           <t>wunde_31</t>
         </is>
       </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="D32" s="9" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
       </c>
-      <c r="E32" s="10" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -4446,22 +4455,22 @@
           <t>wunde_37</t>
         </is>
       </c>
-      <c r="B38" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C38" s="9" t="inlineStr">
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
       </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="E38" s="10" t="inlineStr">
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -4513,22 +4522,22 @@
           <t>wunde_38</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C39" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="D39" s="9" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
       </c>
-      <c r="E39" s="10" t="inlineStr">
+      <c r="E39" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -4580,22 +4589,22 @@
           <t>wunde_39</t>
         </is>
       </c>
-      <c r="B40" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="D40" s="9" t="inlineStr">
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
       </c>
-      <c r="E40" s="10" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -4714,22 +4723,22 @@
           <t>wunde_41</t>
         </is>
       </c>
-      <c r="B42" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C42" s="9" t="inlineStr">
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
       </c>
-      <c r="D42" s="9" t="inlineStr">
+      <c r="D42" s="10" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
       </c>
-      <c r="E42" s="10" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -4781,22 +4790,22 @@
           <t>wunde_42</t>
         </is>
       </c>
-      <c r="B43" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C43" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="D43" s="9" t="inlineStr">
-        <is>
-          <t>Dekubitus</t>
-        </is>
-      </c>
-      <c r="E43" s="10" t="inlineStr">
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>Dekubitus</t>
+        </is>
+      </c>
+      <c r="E43" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -4915,22 +4924,22 @@
           <t>wunde_44</t>
         </is>
       </c>
-      <c r="B45" s="9" t="inlineStr">
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>Ulcus cruris mixtum</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="D45" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="E45" s="10" t="inlineStr">
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="E45" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -4982,22 +4991,22 @@
           <t>wunde_45</t>
         </is>
       </c>
-      <c r="B46" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="D46" s="9" t="inlineStr">
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
       </c>
-      <c r="E46" s="10" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -5116,22 +5125,22 @@
           <t>wunde_47</t>
         </is>
       </c>
-      <c r="B48" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="D48" s="9" t="inlineStr">
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
       </c>
-      <c r="E48" s="10" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -5183,22 +5192,22 @@
           <t>wunde_48</t>
         </is>
       </c>
-      <c r="B49" s="9" t="inlineStr">
-        <is>
-          <t>Dekubitus</t>
-        </is>
-      </c>
-      <c r="C49" s="9" t="inlineStr">
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>Dekubitus</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
       </c>
-      <c r="D49" s="9" t="inlineStr">
+      <c r="D49" s="10" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
       </c>
-      <c r="E49" s="10" t="inlineStr">
+      <c r="E49" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -5384,22 +5393,22 @@
           <t>wunde_51</t>
         </is>
       </c>
-      <c r="B52" s="9" t="inlineStr">
-        <is>
-          <t>Ulkus (Ätiologie unspezifisch)</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>Dekubitus</t>
-        </is>
-      </c>
-      <c r="D52" s="9" t="inlineStr">
-        <is>
-          <t>Dekubitus</t>
-        </is>
-      </c>
-      <c r="E52" s="10" t="inlineStr">
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>Ulkus (Ätiologie unspezifisch)</t>
+        </is>
+      </c>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>Dekubitus</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>Dekubitus</t>
+        </is>
+      </c>
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>2/3 Einig</t>
         </is>
@@ -6050,22 +6059,22 @@
     </row>
     <row r="62"/>
     <row r="63">
-      <c r="A63" s="11" t="inlineStr">
-        <is>
-          <t>STATISTIK &amp; KI-TREFFERQUOTE BEI EXPERTEN (GESAMT 60 WUNDEN &amp; 30 KONSENS-WUNDEN)</t>
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t>STATISTIK &amp; KI-TREFFERQUOTE BEI EXPERTEN (GESAMT 60 WUNDEN, TEILEINIGKEIT &amp; KONSENS-WUNDEN)</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="12" t="inlineStr">
-        <is>
-          <t>KI-Trefferquote Gesamt (vs. jeweilige Experten bei 60 Wunden)</t>
-        </is>
-      </c>
-      <c r="B64" s="13" t="inlineStr"/>
-      <c r="C64" s="13" t="inlineStr"/>
-      <c r="D64" s="13" t="inlineStr"/>
-      <c r="E64" s="13" t="inlineStr"/>
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>KI-Trefferquote Gesamt (vs. jeweilige Experten)</t>
+        </is>
+      </c>
+      <c r="B64" s="14" t="inlineStr"/>
+      <c r="C64" s="14" t="inlineStr"/>
+      <c r="D64" s="14" t="inlineStr"/>
+      <c r="E64" s="14" t="inlineStr"/>
       <c r="F64" s="6" t="inlineStr">
         <is>
           <t>26 / 60 (43.3%)</t>
@@ -6073,7 +6082,7 @@
       </c>
       <c r="G64" s="6" t="inlineStr">
         <is>
-          <t>26 / 60 (43.3%)</t>
+          <t>26 / 58 (44.8%)</t>
         </is>
       </c>
       <c r="H64" s="6" t="inlineStr">
@@ -6081,7 +6090,7 @@
           <t>29 / 60 (48.3%)</t>
         </is>
       </c>
-      <c r="I64" s="14" t="inlineStr">
+      <c r="I64" s="15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6093,7 +6102,7 @@
       </c>
       <c r="K64" s="6" t="inlineStr">
         <is>
-          <t>40 / 60 (66.7%)</t>
+          <t>40 / 58 (69.0%)</t>
         </is>
       </c>
       <c r="L64" s="6" t="inlineStr">
@@ -6101,58 +6110,109 @@
           <t>39 / 60 (65.0%)</t>
         </is>
       </c>
-      <c r="M64" s="14" t="inlineStr">
+      <c r="M64" s="15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="12" t="inlineStr">
-        <is>
-          <t>KI-Trefferquote bei 100% Einigkeit (3/3 = 30 Konsens-Wunden)</t>
-        </is>
-      </c>
-      <c r="B65" s="13" t="inlineStr"/>
-      <c r="C65" s="13" t="inlineStr"/>
-      <c r="D65" s="13" t="inlineStr"/>
-      <c r="E65" s="13" t="inlineStr"/>
+      <c r="A65" s="13" t="inlineStr">
+        <is>
+          <t>KI-Trefferquote bei Teileinigkeit / Mehrheit (2/3 &amp; 3/3)</t>
+        </is>
+      </c>
+      <c r="B65" s="14" t="inlineStr"/>
+      <c r="C65" s="14" t="inlineStr"/>
+      <c r="D65" s="14" t="inlineStr"/>
+      <c r="E65" s="14" t="inlineStr"/>
       <c r="F65" s="6" t="inlineStr">
         <is>
+          <t>18 / 52 (34.6%)</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>19 / 50 (38.0%)</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>20 / 52 (38.5%)</t>
+        </is>
+      </c>
+      <c r="I65" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J65" s="6" t="inlineStr">
+        <is>
+          <t>32 / 52 (61.5%)</t>
+        </is>
+      </c>
+      <c r="K65" s="6" t="inlineStr">
+        <is>
+          <t>36 / 51 (70.6%)</t>
+        </is>
+      </c>
+      <c r="L65" s="6" t="inlineStr">
+        <is>
+          <t>36 / 52 (69.2%)</t>
+        </is>
+      </c>
+      <c r="M65" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="13" t="inlineStr">
+        <is>
+          <t>KI-Trefferquote bei 100% Einigkeit (3/3 Konsens)</t>
+        </is>
+      </c>
+      <c r="B66" s="14" t="inlineStr"/>
+      <c r="C66" s="14" t="inlineStr"/>
+      <c r="D66" s="14" t="inlineStr"/>
+      <c r="E66" s="14" t="inlineStr"/>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
           <t>16 / 30 (53.3%)</t>
         </is>
       </c>
-      <c r="G65" s="6" t="inlineStr">
+      <c r="G66" s="6" t="inlineStr">
         <is>
           <t>16 / 30 (53.3%)</t>
         </is>
       </c>
-      <c r="H65" s="6" t="inlineStr">
+      <c r="H66" s="6" t="inlineStr">
         <is>
           <t>16 / 30 (53.3%)</t>
         </is>
       </c>
-      <c r="I65" s="14" t="inlineStr">
+      <c r="I66" s="15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J65" s="6" t="inlineStr">
+      <c r="J66" s="6" t="inlineStr">
         <is>
           <t>20 / 30 (66.7%)</t>
         </is>
       </c>
-      <c r="K65" s="6" t="inlineStr">
+      <c r="K66" s="6" t="inlineStr">
         <is>
           <t>26 / 30 (86.7%)</t>
         </is>
       </c>
-      <c r="L65" s="6" t="inlineStr">
+      <c r="L66" s="6" t="inlineStr">
         <is>
           <t>23 / 30 (76.7%)</t>
         </is>
       </c>
-      <c r="M65" s="14" t="inlineStr">
+      <c r="M66" s="15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6182,29 +6242,29 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Ziel-Kategorie (Wundtyp-Schema)</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Roh-Eingabe / Originaler Freitext</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="16" t="inlineStr">
         <is>
           <t>Herkunft</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="16" t="inlineStr">
         <is>
           <t>Mapping-Regel / Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>Ausgedehnte feuchte Nekrose</t>
         </is>
@@ -6219,14 +6279,14 @@
           <t>Experte 1 (L&amp;R Raw)</t>
         </is>
       </c>
-      <c r="D2" s="17" t="inlineStr">
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6248,7 +6308,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6270,7 +6330,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6292,7 +6352,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6314,7 +6374,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6336,7 +6396,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6358,7 +6418,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6381,7 +6441,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6403,7 +6463,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6426,7 +6486,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6449,7 +6509,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6472,7 +6532,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6495,7 +6555,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6517,7 +6577,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6539,7 +6599,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6561,7 +6621,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6583,7 +6643,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6605,7 +6665,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6627,7 +6687,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6649,7 +6709,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6671,7 +6731,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6693,7 +6753,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6715,7 +6775,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6737,7 +6797,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6759,7 +6819,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6781,7 +6841,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6803,7 +6863,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6825,7 +6885,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6847,7 +6907,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6869,7 +6929,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6891,7 +6951,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6916,7 +6976,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6938,7 +6998,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+      <c r="A35" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6960,7 +7020,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="16" t="inlineStr">
+      <c r="A36" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -6983,7 +7043,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="inlineStr">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7006,7 +7066,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7028,7 +7088,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="inlineStr">
+      <c r="A39" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7050,7 +7110,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="inlineStr">
+      <c r="A40" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7072,7 +7132,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="16" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7094,7 +7154,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="16" t="inlineStr">
+      <c r="A42" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7116,7 +7176,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="16" t="inlineStr">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7140,7 +7200,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="16" t="inlineStr">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7162,7 +7222,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7185,7 +7245,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="16" t="inlineStr">
+      <c r="A46" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7207,7 +7267,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="16" t="inlineStr">
+      <c r="A47" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7229,7 +7289,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="16" t="inlineStr">
+      <c r="A48" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7251,7 +7311,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="16" t="inlineStr">
+      <c r="A49" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7273,7 +7333,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="16" t="inlineStr">
+      <c r="A50" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7295,7 +7355,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="16" t="inlineStr">
+      <c r="A51" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7317,7 +7377,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="16" t="inlineStr">
+      <c r="A52" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7339,7 +7399,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="16" t="inlineStr">
+      <c r="A53" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7361,7 +7421,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="16" t="inlineStr">
+      <c r="A54" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7383,7 +7443,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="16" t="inlineStr">
+      <c r="A55" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7405,7 +7465,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="16" t="inlineStr">
+      <c r="A56" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7427,7 +7487,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="16" t="inlineStr">
+      <c r="A57" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7449,7 +7509,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="16" t="inlineStr">
+      <c r="A58" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7471,7 +7531,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="16" t="inlineStr">
+      <c r="A59" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7493,7 +7553,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="16" t="inlineStr">
+      <c r="A60" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7515,7 +7575,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="16" t="inlineStr">
+      <c r="A61" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7537,7 +7597,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="16" t="inlineStr">
+      <c r="A62" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7559,7 +7619,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="16" t="inlineStr">
+      <c r="A63" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7581,7 +7641,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="16" t="inlineStr">
+      <c r="A64" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7603,7 +7663,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="16" t="inlineStr">
+      <c r="A65" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7625,7 +7685,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="16" t="inlineStr">
+      <c r="A66" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7647,7 +7707,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="16" t="inlineStr">
+      <c r="A67" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7669,7 +7729,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="16" t="inlineStr">
+      <c r="A68" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7691,7 +7751,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="16" t="inlineStr">
+      <c r="A69" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7713,7 +7773,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="16" t="inlineStr">
+      <c r="A70" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7735,7 +7795,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="16" t="inlineStr">
+      <c r="A71" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7757,7 +7817,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="16" t="inlineStr">
+      <c r="A72" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7779,7 +7839,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="16" t="inlineStr">
+      <c r="A73" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7801,7 +7861,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="16" t="inlineStr">
+      <c r="A74" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7823,7 +7883,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="16" t="inlineStr">
+      <c r="A75" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7845,7 +7905,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="16" t="inlineStr">
+      <c r="A76" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7867,7 +7927,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="16" t="inlineStr">
+      <c r="A77" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7889,7 +7949,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="16" t="inlineStr">
+      <c r="A78" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7911,7 +7971,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="16" t="inlineStr">
+      <c r="A79" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7933,7 +7993,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="16" t="inlineStr">
+      <c r="A80" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7955,7 +8015,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="16" t="inlineStr">
+      <c r="A81" s="17" t="inlineStr">
         <is>
           <t>Dekubitus</t>
         </is>
@@ -7977,7 +8037,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="16" t="inlineStr">
+      <c r="A82" s="17" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
@@ -7999,7 +8059,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="16" t="inlineStr">
+      <c r="A83" s="17" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
@@ -8021,7 +8081,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="16" t="inlineStr">
+      <c r="A84" s="17" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
@@ -8045,7 +8105,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="16" t="inlineStr">
+      <c r="A85" s="17" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
@@ -8067,7 +8127,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="16" t="inlineStr">
+      <c r="A86" s="17" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
@@ -8089,7 +8149,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="16" t="inlineStr">
+      <c r="A87" s="17" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
@@ -8111,7 +8171,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="16" t="inlineStr">
+      <c r="A88" s="17" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
@@ -8133,7 +8193,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="16" t="inlineStr">
+      <c r="A89" s="17" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
@@ -8155,7 +8215,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="16" t="inlineStr">
+      <c r="A90" s="17" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
@@ -8177,7 +8237,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="16" t="inlineStr">
+      <c r="A91" s="17" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
@@ -8199,7 +8259,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="16" t="inlineStr">
+      <c r="A92" s="17" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
@@ -8221,7 +8281,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="16" t="inlineStr">
+      <c r="A93" s="17" t="inlineStr">
         <is>
           <t>Diabetisches Fußsyndrom (DFS)</t>
         </is>
@@ -8243,7 +8303,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="16" t="inlineStr">
+      <c r="A94" s="17" t="inlineStr">
         <is>
           <t>Enthaltung / keine Angabe</t>
         </is>
@@ -8265,7 +8325,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="16" t="inlineStr">
+      <c r="A95" s="17" t="inlineStr">
         <is>
           <t>Enthaltung / keine Angabe</t>
         </is>
@@ -8287,7 +8347,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="16" t="inlineStr">
+      <c r="A96" s="17" t="inlineStr">
         <is>
           <t>Exkoriationen / flächige Erosionen der Hand</t>
         </is>
@@ -8302,14 +8362,14 @@
           <t>Two-Stage L&amp;R KI</t>
         </is>
       </c>
-      <c r="D96" s="17" t="inlineStr">
+      <c r="D96" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="16" t="inlineStr">
+      <c r="A97" s="17" t="inlineStr">
         <is>
           <t>Extravasationsverletzung (Extravasationsverletzung am Fuß/Knöchel eines Säuglings mit ausgeprägter Gewebeschädigung.)</t>
         </is>
@@ -8324,14 +8384,14 @@
           <t>Experte 3 (NursIT Raw)</t>
         </is>
       </c>
-      <c r="D97" s="17" t="inlineStr">
+      <c r="D97" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="16" t="inlineStr">
+      <c r="A98" s="17" t="inlineStr">
         <is>
           <t>Hämangiom ist ein Spezialgebiet. In der Regel ist dieses innerhalb des ersten Lebensjahres rückläufig.
 Deshalb nehme ich hier keine Beurteilung vor.</t>
@@ -8348,14 +8408,14 @@
           <t>Experte 1 (L&amp;R Raw)</t>
         </is>
       </c>
-      <c r="D98" s="17" t="inlineStr">
+      <c r="D98" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="16" t="inlineStr">
+      <c r="A99" s="17" t="inlineStr">
         <is>
           <t>Infizierte Hautläsion / kleiner Abszess</t>
         </is>
@@ -8370,14 +8430,14 @@
           <t>Two-Stage L&amp;R KI</t>
         </is>
       </c>
-      <c r="D99" s="17" t="inlineStr">
+      <c r="D99" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="16" t="inlineStr">
+      <c r="A100" s="17" t="inlineStr">
         <is>
           <t>Infizierte Wunden am linken Oberarm / Innenseitig</t>
         </is>
@@ -8392,14 +8452,14 @@
           <t>Experte 1 (L&amp;R Raw)</t>
         </is>
       </c>
-      <c r="D100" s="17" t="inlineStr">
+      <c r="D100" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="16" t="inlineStr">
+      <c r="A101" s="17" t="inlineStr">
         <is>
           <t>Kleiner Abszess/Sinusöffnung (infizierte oberflächliche Hautläsion)</t>
         </is>
@@ -8414,14 +8474,14 @@
           <t>Zero-Shot L&amp;R KI</t>
         </is>
       </c>
-      <c r="D101" s="17" t="inlineStr">
+      <c r="D101" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="16" t="inlineStr">
+      <c r="A102" s="17" t="inlineStr">
         <is>
           <t>Pilonidalsinus (Sinus pilonidalis)</t>
         </is>
@@ -8436,14 +8496,14 @@
           <t>Two-Stage L&amp;R KI</t>
         </is>
       </c>
-      <c r="D102" s="17" t="inlineStr">
+      <c r="D102" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="16" t="inlineStr">
+      <c r="A103" s="17" t="inlineStr">
         <is>
           <t>Plantares Ulcus linker Fuß, Ursachen Klärung notwendig, bei Diabetiker Prüfung ob Neuropathisch oder Angiopathische Ursache</t>
         </is>
@@ -8458,14 +8518,14 @@
           <t>Experte 2 (L&amp;R Raw)</t>
         </is>
       </c>
-      <c r="D103" s="17" t="inlineStr">
+      <c r="D103" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="16" t="inlineStr">
+      <c r="A104" s="17" t="inlineStr">
         <is>
           <t>Postoperative Wunde / Dehiszenz</t>
         </is>
@@ -8487,7 +8547,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="16" t="inlineStr">
+      <c r="A105" s="17" t="inlineStr">
         <is>
           <t>Postoperative Wunde / Dehiszenz</t>
         </is>
@@ -8509,7 +8569,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="16" t="inlineStr">
+      <c r="A106" s="17" t="inlineStr">
         <is>
           <t>Postoperative Wunde / Dehiszenz</t>
         </is>
@@ -8531,7 +8591,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="16" t="inlineStr">
+      <c r="A107" s="17" t="inlineStr">
         <is>
           <t>Postoperative Wunde / Dehiszenz</t>
         </is>
@@ -8553,7 +8613,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="16" t="inlineStr">
+      <c r="A108" s="17" t="inlineStr">
         <is>
           <t>Postoperative Wunde / Dehiszenz</t>
         </is>
@@ -8575,7 +8635,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="16" t="inlineStr">
+      <c r="A109" s="17" t="inlineStr">
         <is>
           <t>Postoperative Wunde / Dehiszenz</t>
         </is>
@@ -8597,7 +8657,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="16" t="inlineStr">
+      <c r="A110" s="17" t="inlineStr">
         <is>
           <t>Postoperative Wunde / Dehiszenz</t>
         </is>
@@ -8619,7 +8679,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="16" t="inlineStr">
+      <c r="A111" s="17" t="inlineStr">
         <is>
           <t>Postoperative Wunde / Dehiszenz</t>
         </is>
@@ -8641,7 +8701,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="16" t="inlineStr">
+      <c r="A112" s="17" t="inlineStr">
         <is>
           <t>Postoperative Wunde / Dehiszenz</t>
         </is>
@@ -8663,7 +8723,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="16" t="inlineStr">
+      <c r="A113" s="17" t="inlineStr">
         <is>
           <t>Postoperative Wunde / Dehiszenz</t>
         </is>
@@ -8685,7 +8745,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="16" t="inlineStr">
+      <c r="A114" s="17" t="inlineStr">
         <is>
           <t>Reibungsblase / oberflächliche Hautläsion</t>
         </is>
@@ -8700,14 +8760,14 @@
           <t>Few-Shot L&amp;R KI</t>
         </is>
       </c>
-      <c r="D114" s="17" t="inlineStr">
+      <c r="D114" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="16" t="inlineStr">
+      <c r="A115" s="17" t="inlineStr">
         <is>
           <t>Traumatische Wunde</t>
         </is>
@@ -8729,7 +8789,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="16" t="inlineStr">
+      <c r="A116" s="17" t="inlineStr">
         <is>
           <t>Traumatische Wunde</t>
         </is>
@@ -8751,7 +8811,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="16" t="inlineStr">
+      <c r="A117" s="17" t="inlineStr">
         <is>
           <t>Traumatische Wunde</t>
         </is>
@@ -8773,7 +8833,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="16" t="inlineStr">
+      <c r="A118" s="17" t="inlineStr">
         <is>
           <t>Traumatische Wunde</t>
         </is>
@@ -8795,7 +8855,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="16" t="inlineStr">
+      <c r="A119" s="17" t="inlineStr">
         <is>
           <t>Traumatische Wunde</t>
         </is>
@@ -8817,7 +8877,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="16" t="inlineStr">
+      <c r="A120" s="17" t="inlineStr">
         <is>
           <t>Traumatische Wunde</t>
         </is>
@@ -8843,7 +8903,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="16" t="inlineStr">
+      <c r="A121" s="17" t="inlineStr">
         <is>
           <t>Traumatische Wunde</t>
         </is>
@@ -8865,7 +8925,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="16" t="inlineStr">
+      <c r="A122" s="17" t="inlineStr">
         <is>
           <t>Traumatische Wunde</t>
         </is>
@@ -8887,7 +8947,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="16" t="inlineStr">
+      <c r="A123" s="17" t="inlineStr">
         <is>
           <t>Traumatische Wunde</t>
         </is>
@@ -8909,7 +8969,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="16" t="inlineStr">
+      <c r="A124" s="17" t="inlineStr">
         <is>
           <t>Traumatische Wunde</t>
         </is>
@@ -8931,7 +8991,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="16" t="inlineStr">
+      <c r="A125" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
@@ -8953,7 +9013,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="16" t="inlineStr">
+      <c r="A126" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
@@ -8975,7 +9035,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="16" t="inlineStr">
+      <c r="A127" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
@@ -8997,7 +9057,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="16" t="inlineStr">
+      <c r="A128" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
@@ -9019,7 +9079,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="16" t="inlineStr">
+      <c r="A129" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
@@ -9041,7 +9101,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="16" t="inlineStr">
+      <c r="A130" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
@@ -9063,7 +9123,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="16" t="inlineStr">
+      <c r="A131" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
@@ -9085,7 +9145,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="16" t="inlineStr">
+      <c r="A132" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
@@ -9107,7 +9167,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="16" t="inlineStr">
+      <c r="A133" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
@@ -9129,7 +9189,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="16" t="inlineStr">
+      <c r="A134" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
@@ -9151,7 +9211,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="16" t="inlineStr">
+      <c r="A135" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
@@ -9173,7 +9233,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="16" t="inlineStr">
+      <c r="A136" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris arteriosum / Ischämisches Ulkus</t>
         </is>
@@ -9196,7 +9256,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="16" t="inlineStr">
+      <c r="A137" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris mixtum</t>
         </is>
@@ -9218,7 +9278,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="16" t="inlineStr">
+      <c r="A138" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris mixtum</t>
         </is>
@@ -9241,7 +9301,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="16" t="inlineStr">
+      <c r="A139" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris mixtum</t>
         </is>
@@ -9263,7 +9323,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="16" t="inlineStr">
+      <c r="A140" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9285,7 +9345,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="16" t="inlineStr">
+      <c r="A141" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9307,7 +9367,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="16" t="inlineStr">
+      <c r="A142" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9329,7 +9389,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="16" t="inlineStr">
+      <c r="A143" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9351,7 +9411,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="16" t="inlineStr">
+      <c r="A144" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9373,7 +9433,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="16" t="inlineStr">
+      <c r="A145" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9395,7 +9455,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="16" t="inlineStr">
+      <c r="A146" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9417,7 +9477,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="16" t="inlineStr">
+      <c r="A147" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9439,7 +9499,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="16" t="inlineStr">
+      <c r="A148" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9461,7 +9521,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="16" t="inlineStr">
+      <c r="A149" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9483,7 +9543,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="16" t="inlineStr">
+      <c r="A150" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9505,7 +9565,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="16" t="inlineStr">
+      <c r="A151" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9527,7 +9587,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="16" t="inlineStr">
+      <c r="A152" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9549,7 +9609,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="16" t="inlineStr">
+      <c r="A153" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9572,7 +9632,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="16" t="inlineStr">
+      <c r="A154" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9594,7 +9654,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="16" t="inlineStr">
+      <c r="A155" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9616,7 +9676,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="16" t="inlineStr">
+      <c r="A156" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9638,7 +9698,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="16" t="inlineStr">
+      <c r="A157" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9660,7 +9720,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="16" t="inlineStr">
+      <c r="A158" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9682,7 +9742,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="16" t="inlineStr">
+      <c r="A159" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9706,7 +9766,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="16" t="inlineStr">
+      <c r="A160" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9728,7 +9788,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="16" t="inlineStr">
+      <c r="A161" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9750,7 +9810,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="16" t="inlineStr">
+      <c r="A162" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9773,7 +9833,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="16" t="inlineStr">
+      <c r="A163" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9798,7 +9858,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="16" t="inlineStr">
+      <c r="A164" s="17" t="inlineStr">
         <is>
           <t>Ulcus cruris venosum</t>
         </is>
@@ -9820,7 +9880,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="16" t="inlineStr">
+      <c r="A165" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -9842,7 +9902,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="16" t="inlineStr">
+      <c r="A166" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -9864,7 +9924,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="16" t="inlineStr">
+      <c r="A167" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -9886,7 +9946,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="16" t="inlineStr">
+      <c r="A168" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -9908,7 +9968,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="16" t="inlineStr">
+      <c r="A169" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -9930,7 +9990,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="16" t="inlineStr">
+      <c r="A170" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -9952,7 +10012,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="16" t="inlineStr">
+      <c r="A171" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -9974,7 +10034,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="16" t="inlineStr">
+      <c r="A172" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -9996,7 +10056,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="16" t="inlineStr">
+      <c r="A173" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10018,7 +10078,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="16" t="inlineStr">
+      <c r="A174" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10040,7 +10100,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="16" t="inlineStr">
+      <c r="A175" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10062,7 +10122,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="16" t="inlineStr">
+      <c r="A176" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10084,7 +10144,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="16" t="inlineStr">
+      <c r="A177" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10106,7 +10166,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="16" t="inlineStr">
+      <c r="A178" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10128,7 +10188,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="16" t="inlineStr">
+      <c r="A179" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10150,7 +10210,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="16" t="inlineStr">
+      <c r="A180" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10172,7 +10232,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="16" t="inlineStr">
+      <c r="A181" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10194,7 +10254,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="16" t="inlineStr">
+      <c r="A182" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10216,7 +10276,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="16" t="inlineStr">
+      <c r="A183" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10238,7 +10298,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="16" t="inlineStr">
+      <c r="A184" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10260,7 +10320,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="16" t="inlineStr">
+      <c r="A185" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10282,7 +10342,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="16" t="inlineStr">
+      <c r="A186" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10304,7 +10364,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="16" t="inlineStr">
+      <c r="A187" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10326,7 +10386,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="16" t="inlineStr">
+      <c r="A188" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10348,7 +10408,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="16" t="inlineStr">
+      <c r="A189" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10370,7 +10430,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="16" t="inlineStr">
+      <c r="A190" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10392,7 +10452,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="16" t="inlineStr">
+      <c r="A191" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10414,7 +10474,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="16" t="inlineStr">
+      <c r="A192" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10436,7 +10496,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="16" t="inlineStr">
+      <c r="A193" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10458,7 +10518,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="16" t="inlineStr">
+      <c r="A194" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10480,7 +10540,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="16" t="inlineStr">
+      <c r="A195" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10502,7 +10562,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="16" t="inlineStr">
+      <c r="A196" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10524,7 +10584,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="16" t="inlineStr">
+      <c r="A197" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10546,7 +10606,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="16" t="inlineStr">
+      <c r="A198" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10568,7 +10628,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="16" t="inlineStr">
+      <c r="A199" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10590,7 +10650,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="16" t="inlineStr">
+      <c r="A200" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10612,7 +10672,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="16" t="inlineStr">
+      <c r="A201" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10635,7 +10695,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="16" t="inlineStr">
+      <c r="A202" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10657,7 +10717,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="16" t="inlineStr">
+      <c r="A203" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10679,7 +10739,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="16" t="inlineStr">
+      <c r="A204" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10701,7 +10761,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="16" t="inlineStr">
+      <c r="A205" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10723,7 +10783,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="16" t="inlineStr">
+      <c r="A206" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10745,7 +10805,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="16" t="inlineStr">
+      <c r="A207" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10767,7 +10827,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="16" t="inlineStr">
+      <c r="A208" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10789,7 +10849,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="16" t="inlineStr">
+      <c r="A209" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10811,7 +10871,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="16" t="inlineStr">
+      <c r="A210" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10833,7 +10893,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="16" t="inlineStr">
+      <c r="A211" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10855,7 +10915,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="16" t="inlineStr">
+      <c r="A212" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10877,7 +10937,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="16" t="inlineStr">
+      <c r="A213" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10899,7 +10959,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="16" t="inlineStr">
+      <c r="A214" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10921,7 +10981,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="16" t="inlineStr">
+      <c r="A215" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10943,7 +11003,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="16" t="inlineStr">
+      <c r="A216" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10965,7 +11025,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="16" t="inlineStr">
+      <c r="A217" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -10987,7 +11047,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="16" t="inlineStr">
+      <c r="A218" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11009,7 +11069,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="16" t="inlineStr">
+      <c r="A219" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11031,7 +11091,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="16" t="inlineStr">
+      <c r="A220" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11053,7 +11113,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="16" t="inlineStr">
+      <c r="A221" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11075,7 +11135,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="16" t="inlineStr">
+      <c r="A222" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11097,7 +11157,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="16" t="inlineStr">
+      <c r="A223" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11119,7 +11179,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="16" t="inlineStr">
+      <c r="A224" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11141,7 +11201,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="16" t="inlineStr">
+      <c r="A225" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11163,7 +11223,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="16" t="inlineStr">
+      <c r="A226" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11185,7 +11245,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="16" t="inlineStr">
+      <c r="A227" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11207,7 +11267,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="16" t="inlineStr">
+      <c r="A228" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11229,7 +11289,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="16" t="inlineStr">
+      <c r="A229" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11251,7 +11311,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="16" t="inlineStr">
+      <c r="A230" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11273,7 +11333,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="16" t="inlineStr">
+      <c r="A231" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11295,7 +11355,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="16" t="inlineStr">
+      <c r="A232" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11317,7 +11377,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="16" t="inlineStr">
+      <c r="A233" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11339,7 +11399,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="16" t="inlineStr">
+      <c r="A234" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11361,7 +11421,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="16" t="inlineStr">
+      <c r="A235" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11383,7 +11443,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="16" t="inlineStr">
+      <c r="A236" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11405,7 +11465,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="16" t="inlineStr">
+      <c r="A237" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11427,7 +11487,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="16" t="inlineStr">
+      <c r="A238" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11449,7 +11509,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="16" t="inlineStr">
+      <c r="A239" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11471,7 +11531,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="16" t="inlineStr">
+      <c r="A240" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11493,7 +11553,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="16" t="inlineStr">
+      <c r="A241" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11515,7 +11575,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="16" t="inlineStr">
+      <c r="A242" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11537,7 +11597,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="16" t="inlineStr">
+      <c r="A243" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11560,7 +11620,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="16" t="inlineStr">
+      <c r="A244" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11582,7 +11642,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="16" t="inlineStr">
+      <c r="A245" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11604,7 +11664,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="16" t="inlineStr">
+      <c r="A246" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11626,7 +11686,7 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="16" t="inlineStr">
+      <c r="A247" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11648,7 +11708,7 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="16" t="inlineStr">
+      <c r="A248" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11671,7 +11731,7 @@
       </c>
     </row>
     <row r="249">
-      <c r="A249" s="16" t="inlineStr">
+      <c r="A249" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11693,7 +11753,7 @@
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="16" t="inlineStr">
+      <c r="A250" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11715,7 +11775,7 @@
       </c>
     </row>
     <row r="251">
-      <c r="A251" s="16" t="inlineStr">
+      <c r="A251" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11737,7 +11797,7 @@
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="16" t="inlineStr">
+      <c r="A252" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11759,7 +11819,7 @@
       </c>
     </row>
     <row r="253">
-      <c r="A253" s="16" t="inlineStr">
+      <c r="A253" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11781,7 +11841,7 @@
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="16" t="inlineStr">
+      <c r="A254" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11803,7 +11863,7 @@
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="16" t="inlineStr">
+      <c r="A255" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11825,7 +11885,7 @@
       </c>
     </row>
     <row r="256">
-      <c r="A256" s="16" t="inlineStr">
+      <c r="A256" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11847,7 +11907,7 @@
       </c>
     </row>
     <row r="257">
-      <c r="A257" s="16" t="inlineStr">
+      <c r="A257" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11869,7 +11929,7 @@
       </c>
     </row>
     <row r="258">
-      <c r="A258" s="16" t="inlineStr">
+      <c r="A258" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11891,7 +11951,7 @@
       </c>
     </row>
     <row r="259">
-      <c r="A259" s="16" t="inlineStr">
+      <c r="A259" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11913,7 +11973,7 @@
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="16" t="inlineStr">
+      <c r="A260" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11935,7 +11995,7 @@
       </c>
     </row>
     <row r="261">
-      <c r="A261" s="16" t="inlineStr">
+      <c r="A261" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11957,7 +12017,7 @@
       </c>
     </row>
     <row r="262">
-      <c r="A262" s="16" t="inlineStr">
+      <c r="A262" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -11979,7 +12039,7 @@
       </c>
     </row>
     <row r="263">
-      <c r="A263" s="16" t="inlineStr">
+      <c r="A263" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12001,7 +12061,7 @@
       </c>
     </row>
     <row r="264">
-      <c r="A264" s="16" t="inlineStr">
+      <c r="A264" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12023,7 +12083,7 @@
       </c>
     </row>
     <row r="265">
-      <c r="A265" s="16" t="inlineStr">
+      <c r="A265" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12045,7 +12105,7 @@
       </c>
     </row>
     <row r="266">
-      <c r="A266" s="16" t="inlineStr">
+      <c r="A266" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12067,7 +12127,7 @@
       </c>
     </row>
     <row r="267">
-      <c r="A267" s="16" t="inlineStr">
+      <c r="A267" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12089,7 +12149,7 @@
       </c>
     </row>
     <row r="268">
-      <c r="A268" s="16" t="inlineStr">
+      <c r="A268" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12111,7 +12171,7 @@
       </c>
     </row>
     <row r="269">
-      <c r="A269" s="16" t="inlineStr">
+      <c r="A269" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12133,7 +12193,7 @@
       </c>
     </row>
     <row r="270">
-      <c r="A270" s="16" t="inlineStr">
+      <c r="A270" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12155,7 +12215,7 @@
       </c>
     </row>
     <row r="271">
-      <c r="A271" s="16" t="inlineStr">
+      <c r="A271" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12177,7 +12237,7 @@
       </c>
     </row>
     <row r="272">
-      <c r="A272" s="16" t="inlineStr">
+      <c r="A272" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12199,7 +12259,7 @@
       </c>
     </row>
     <row r="273">
-      <c r="A273" s="16" t="inlineStr">
+      <c r="A273" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12221,7 +12281,7 @@
       </c>
     </row>
     <row r="274">
-      <c r="A274" s="16" t="inlineStr">
+      <c r="A274" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12243,7 +12303,7 @@
       </c>
     </row>
     <row r="275">
-      <c r="A275" s="16" t="inlineStr">
+      <c r="A275" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12266,7 +12326,7 @@
       </c>
     </row>
     <row r="276">
-      <c r="A276" s="16" t="inlineStr">
+      <c r="A276" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12288,7 +12348,7 @@
       </c>
     </row>
     <row r="277">
-      <c r="A277" s="16" t="inlineStr">
+      <c r="A277" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12310,7 +12370,7 @@
       </c>
     </row>
     <row r="278">
-      <c r="A278" s="16" t="inlineStr">
+      <c r="A278" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12332,7 +12392,7 @@
       </c>
     </row>
     <row r="279">
-      <c r="A279" s="16" t="inlineStr">
+      <c r="A279" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12354,7 +12414,7 @@
       </c>
     </row>
     <row r="280">
-      <c r="A280" s="16" t="inlineStr">
+      <c r="A280" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12376,7 +12436,7 @@
       </c>
     </row>
     <row r="281">
-      <c r="A281" s="16" t="inlineStr">
+      <c r="A281" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12398,7 +12458,7 @@
       </c>
     </row>
     <row r="282">
-      <c r="A282" s="16" t="inlineStr">
+      <c r="A282" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12421,7 +12481,7 @@
       </c>
     </row>
     <row r="283">
-      <c r="A283" s="16" t="inlineStr">
+      <c r="A283" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12443,7 +12503,7 @@
       </c>
     </row>
     <row r="284">
-      <c r="A284" s="16" t="inlineStr">
+      <c r="A284" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12465,7 +12525,7 @@
       </c>
     </row>
     <row r="285">
-      <c r="A285" s="16" t="inlineStr">
+      <c r="A285" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12487,7 +12547,7 @@
       </c>
     </row>
     <row r="286">
-      <c r="A286" s="16" t="inlineStr">
+      <c r="A286" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12509,7 +12569,7 @@
       </c>
     </row>
     <row r="287">
-      <c r="A287" s="16" t="inlineStr">
+      <c r="A287" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12531,7 +12591,7 @@
       </c>
     </row>
     <row r="288">
-      <c r="A288" s="16" t="inlineStr">
+      <c r="A288" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12553,7 +12613,7 @@
       </c>
     </row>
     <row r="289">
-      <c r="A289" s="16" t="inlineStr">
+      <c r="A289" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12575,7 +12635,7 @@
       </c>
     </row>
     <row r="290">
-      <c r="A290" s="16" t="inlineStr">
+      <c r="A290" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12597,7 +12657,7 @@
       </c>
     </row>
     <row r="291">
-      <c r="A291" s="16" t="inlineStr">
+      <c r="A291" s="17" t="inlineStr">
         <is>
           <t>Ulkus (Ätiologie unspezifisch)</t>
         </is>
@@ -12625,7 +12685,7 @@
       </c>
     </row>
     <row r="292">
-      <c r="A292" s="16" t="inlineStr">
+      <c r="A292" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12647,7 +12707,7 @@
       </c>
     </row>
     <row r="293">
-      <c r="A293" s="16" t="inlineStr">
+      <c r="A293" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12669,7 +12729,7 @@
       </c>
     </row>
     <row r="294">
-      <c r="A294" s="16" t="inlineStr">
+      <c r="A294" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12691,7 +12751,7 @@
       </c>
     </row>
     <row r="295">
-      <c r="A295" s="16" t="inlineStr">
+      <c r="A295" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12713,7 +12773,7 @@
       </c>
     </row>
     <row r="296">
-      <c r="A296" s="16" t="inlineStr">
+      <c r="A296" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12735,7 +12795,7 @@
       </c>
     </row>
     <row r="297">
-      <c r="A297" s="16" t="inlineStr">
+      <c r="A297" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12757,7 +12817,7 @@
       </c>
     </row>
     <row r="298">
-      <c r="A298" s="16" t="inlineStr">
+      <c r="A298" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12779,7 +12839,7 @@
       </c>
     </row>
     <row r="299">
-      <c r="A299" s="16" t="inlineStr">
+      <c r="A299" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12801,7 +12861,7 @@
       </c>
     </row>
     <row r="300">
-      <c r="A300" s="16" t="inlineStr">
+      <c r="A300" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12823,7 +12883,7 @@
       </c>
     </row>
     <row r="301">
-      <c r="A301" s="16" t="inlineStr">
+      <c r="A301" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12845,7 +12905,7 @@
       </c>
     </row>
     <row r="302">
-      <c r="A302" s="16" t="inlineStr">
+      <c r="A302" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12867,7 +12927,7 @@
       </c>
     </row>
     <row r="303">
-      <c r="A303" s="16" t="inlineStr">
+      <c r="A303" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12889,7 +12949,7 @@
       </c>
     </row>
     <row r="304">
-      <c r="A304" s="16" t="inlineStr">
+      <c r="A304" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12911,7 +12971,7 @@
       </c>
     </row>
     <row r="305">
-      <c r="A305" s="16" t="inlineStr">
+      <c r="A305" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12933,7 +12993,7 @@
       </c>
     </row>
     <row r="306">
-      <c r="A306" s="16" t="inlineStr">
+      <c r="A306" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12955,7 +13015,7 @@
       </c>
     </row>
     <row r="307">
-      <c r="A307" s="16" t="inlineStr">
+      <c r="A307" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -12978,7 +13038,7 @@
       </c>
     </row>
     <row r="308">
-      <c r="A308" s="16" t="inlineStr">
+      <c r="A308" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -13001,7 +13061,7 @@
       </c>
     </row>
     <row r="309">
-      <c r="A309" s="16" t="inlineStr">
+      <c r="A309" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -13023,7 +13083,7 @@
       </c>
     </row>
     <row r="310">
-      <c r="A310" s="16" t="inlineStr">
+      <c r="A310" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -13045,7 +13105,7 @@
       </c>
     </row>
     <row r="311">
-      <c r="A311" s="16" t="inlineStr">
+      <c r="A311" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -13067,7 +13127,7 @@
       </c>
     </row>
     <row r="312">
-      <c r="A312" s="16" t="inlineStr">
+      <c r="A312" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -13089,7 +13149,7 @@
       </c>
     </row>
     <row r="313">
-      <c r="A313" s="16" t="inlineStr">
+      <c r="A313" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -13111,7 +13171,7 @@
       </c>
     </row>
     <row r="314">
-      <c r="A314" s="16" t="inlineStr">
+      <c r="A314" s="17" t="inlineStr">
         <is>
           <t>Verbrennungswunde</t>
         </is>
@@ -13133,7 +13193,7 @@
       </c>
     </row>
     <row r="315">
-      <c r="A315" s="16" t="inlineStr">
+      <c r="A315" s="17" t="inlineStr">
         <is>
           <t>Wunde am li Fußrücken mit Sehnenfreilegung</t>
         </is>
@@ -13148,14 +13208,14 @@
           <t>Experte 1 (L&amp;R Raw)</t>
         </is>
       </c>
-      <c r="D315" s="17" t="inlineStr">
+      <c r="D315" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="316">
-      <c r="A316" s="16" t="inlineStr">
+      <c r="A316" s="17" t="inlineStr">
         <is>
           <t>Wunde aufgrund einer Infusion, welche ins umliegende Gewebe ausgetreten ist</t>
         </is>
@@ -13170,14 +13230,14 @@
           <t>Experte 1 (L&amp;R Raw)</t>
         </is>
       </c>
-      <c r="D316" s="17" t="inlineStr">
+      <c r="D316" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="317">
-      <c r="A317" s="16" t="inlineStr">
+      <c r="A317" s="17" t="inlineStr">
         <is>
           <t>infantiles Hämangiom,</t>
         </is>
@@ -13192,14 +13252,14 @@
           <t>Experte 2 (L&amp;R Raw)</t>
         </is>
       </c>
-      <c r="D317" s="17" t="inlineStr">
+      <c r="D317" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="318">
-      <c r="A318" s="16" t="inlineStr">
+      <c r="A318" s="17" t="inlineStr">
         <is>
           <t>nekrotischen Wunden am Fuß</t>
         </is>
@@ -13214,14 +13274,14 @@
           <t>Experte 1 (L&amp;R Raw)</t>
         </is>
       </c>
-      <c r="D318" s="17" t="inlineStr">
+      <c r="D318" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="319">
-      <c r="A319" s="16" t="inlineStr">
+      <c r="A319" s="17" t="inlineStr">
         <is>
           <t>rechter Fuß lateral/ malleolär</t>
         </is>
@@ -13236,14 +13296,14 @@
           <t>Experte 2 (L&amp;R Raw)</t>
         </is>
       </c>
-      <c r="D319" s="17" t="inlineStr">
+      <c r="D319" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>
       </c>
     </row>
     <row r="320">
-      <c r="A320" s="16" t="inlineStr">
+      <c r="A320" s="17" t="inlineStr">
         <is>
           <t>ulzeriertes infantiles Hämangiom mit zentraler Nekrose (exophytisches, livid-rötliches Hämangiom mit zentralem nekrotisch-fibrinösem Defekt)</t>
         </is>
@@ -13258,7 +13318,7 @@
           <t>Experte 3 (NursIT Raw)</t>
         </is>
       </c>
-      <c r="D320" s="17" t="inlineStr">
+      <c r="D320" s="18" t="inlineStr">
         <is>
           <t>Freitext belassen (Kein Matching)</t>
         </is>

</xml_diff>